<commit_message>
Rechnung RE202606050129 fuer Max Mustermann
</commit_message>
<xml_diff>
--- a/rechnungslog.xlsx
+++ b/rechnungslog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,49 @@
         <v>30</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>05.06.2026 01:30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RE202606050129</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Max Mustermann</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>max@example.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Musterstr. 1, 97070 Wuerzburg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Chipschloss XY</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Diagnose x2, Schloss einbauen x1, Anfahrt x1, Notdienst x1</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>310</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rechnung RE202606050133 fuer Max Mustermann
</commit_message>
<xml_diff>
--- a/rechnungslog.xlsx
+++ b/rechnungslog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -572,6 +572,49 @@
         <v>310</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>05.06.2026 01:33</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RE202606050133</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Max Mustermann</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>max@example.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Musterstr. 1, 97070 Wuerzburg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Chipschloss XY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Diagnose x1, Schloss einbauen x1, Batterietausch x1</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>325</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rechnung RE202606050824 fuer Max Mustermann
</commit_message>
<xml_diff>
--- a/rechnungslog.xlsx
+++ b/rechnungslog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -615,6 +615,49 @@
         <v>325</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>05.06.2026 08:24</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RE202606050824</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Max Mustermann</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>max@example.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Musterstr. 1, 97070 Wuerzburg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Chipschloss XY</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Anfahrt x1, Chip programmieren x1, Batterietausch x1, Schloss einbauen x1</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>240</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rechnung RE202606050941 fuer Max Mustermann
</commit_message>
<xml_diff>
--- a/rechnungslog.xlsx
+++ b/rechnungslog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -658,6 +658,49 @@
         <v>240</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05.06.2026 09:41</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RE202606050941</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Max Mustermann</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>max@example.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Musterstr. 1, 97070 Wuerzburg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Chipschloss XY</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Notdienst x1, Chip programmieren x1, Anfahrt x1, Schloss einbauen x1</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>175</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>